<commit_message>
29.09. Sve je komitovano jer sam ostao sam
</commit_message>
<xml_diff>
--- a/results/TestResults.xlsx
+++ b/results/TestResults.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="51">
   <si>
     <t>App</t>
   </si>
@@ -59,13 +59,13 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Credit_Cards_Details_Card_Details_[WEB]</t>
+    <t>Payments_Domestic_Payments_Internal_Non_Urgent_Payment_[WEB]</t>
   </si>
   <si>
     <t>FAILED</t>
   </si>
   <si>
-    <t>15.09.2026:11:00</t>
+    <t>29.09.2026:08:52</t>
   </si>
   <si>
     <t>dev</t>
@@ -74,46 +74,112 @@
     <t/>
   </si>
   <si>
-    <t>DTC-103</t>
-  </si>
-  <si>
-    <t>Chrome</t>
+    <t>DTC-133</t>
   </si>
   <si>
     <t>Web</t>
   </si>
   <si>
-    <t>Credit_Cards_Details_Card_Details_[WEB]_15_09_2026_11_00.jpg</t>
+    <t>Payments_Domestic_Payments_Internal_Non_Urgent_Payment_[WEB]_29_09_2026_08_52.jpg</t>
   </si>
   <si>
-    <t>Product_Summary-Current_Foreign_Accounts_List_[WEB]</t>
+    <t>29.09.2026:08:53</t>
   </si>
   <si>
-    <t>PASSED</t>
-  </si>
-  <si>
-    <t>22.09.2026:13:12</t>
-  </si>
-  <si>
-    <t>Product_Summary-Current_Domestic_Accounts_List_[WEB]</t>
-  </si>
-  <si>
-    <t>22.09.2026:13:18</t>
+    <t>Payments_Domestic_Payments_Internal_Non_Urgent_Payment_[WEB]_29_09_2026_08_53.jpg</t>
   </si>
   <si>
     <t>Current_Domestic_Accounts-Transactions-Filter_By_Date-Predefined_Date_Range_[WEB]</t>
   </si>
   <si>
-    <t>23.09.2026:06:59</t>
+    <t>29.09.2026:09:04</t>
   </si>
   <si>
-    <t>failed</t>
+    <t>Current_Domestic_Accounts-Transactions-Filter_By_Date-Predefined_Date_Range_[WEB]_29_09_2026_09_04.jpg</t>
   </si>
   <si>
-    <t>23.09.2026:07:00</t>
+    <t>Payments-Payments_Overview_[WEB]</t>
   </si>
   <si>
-    <t>23.09.2026:07:04</t>
+    <t>29.09.2026:09:32</t>
+  </si>
+  <si>
+    <t>Payments-Payments_Overview_[WEB]_29_09_2026_09_32.jpg</t>
+  </si>
+  <si>
+    <t>29.09.2026:09:35</t>
+  </si>
+  <si>
+    <t>Payments-Payments_Overview_[WEB]_29_09_2026_09_35.jpg</t>
+  </si>
+  <si>
+    <t>29.09.2026:09:36</t>
+  </si>
+  <si>
+    <t>Payments-Payments_Overview_[WEB]_29_09_2026_09_36.jpg</t>
+  </si>
+  <si>
+    <t>Payments_Payments_Archive_Payments_Details_[WEB]</t>
+  </si>
+  <si>
+    <t>29.09.2026:09:45</t>
+  </si>
+  <si>
+    <t>Payments_Payments_Archive_Payments_Details_[WEB]_29_09_2026_09_45.jpg</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_External_Urgent_Payment_No_Model_[WEB]</t>
+  </si>
+  <si>
+    <t>29.09.2026:11:03</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_External_Urgent_Payment_No_Model_[WEB]_29_09_2026_11_03.jpg</t>
+  </si>
+  <si>
+    <t>29.09.2026:11:04</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_External_Urgent_Payment_No_Model_[WEB]_29_09_2026_11_04.jpg</t>
+  </si>
+  <si>
+    <t>29.09.2026:11:05</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_External_Urgent_Payment_No_Model_[WEB]_29_09_2026_11_05.jpg</t>
+  </si>
+  <si>
+    <t>Payments_Currency_Exchange_[WEB]-Buy_From_Payment</t>
+  </si>
+  <si>
+    <t>29.09.2026:11:06</t>
+  </si>
+  <si>
+    <t>Payments_Currency_Exchange_[WEB]-Buy_From_Payment_29_09_2026_11_06.jpg</t>
+  </si>
+  <si>
+    <t>29.09.2026:11:13</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_External_Urgent_Payment_No_Model_[WEB]_29_09_2026_11_13.jpg</t>
+  </si>
+  <si>
+    <t>29.09.2026:11:16</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_External_Urgent_Payment_No_Model_[WEB]_29_09_2026_11_16.jpg</t>
+  </si>
+  <si>
+    <t>29.09.2026:11:44</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_External_Urgent_Payment_No_Model_[WEB]_29_09_2026_11_44.jpg</t>
+  </si>
+  <si>
+    <t>29.09.2026:11:49</t>
+  </si>
+  <si>
+    <t>Payments_Domestic_Payments_External_Urgent_Payment_No_Model_[WEB]_29_09_2026_11_49.jpg</t>
   </si>
 </sst>
 </file>
@@ -285,7 +351,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="37">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -490,11 +556,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="10"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="17"/>
       </patternFill>
     </fill>
   </fills>
@@ -769,7 +830,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="147">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -788,24 +849,6 @@
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
@@ -824,15 +867,123 @@
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="true"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2001,7 +2152,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:XFD7"/>
+  <dimension ref="A1:XFD17"/>
   <sheetFormatPr defaultColWidth="8.82407407407407" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col min="1" max="1" customWidth="true" style="1" width="9.33333333333333" collapsed="true"/>
@@ -18444,24 +18595,24 @@
         <v>15</v>
       </c>
       <c r="H2" t="s" s="9">
+        <v>14</v>
+      </c>
+      <c r="I2" t="s" s="10">
         <v>16</v>
       </c>
-      <c r="I2" t="s" s="10">
+      <c r="J2" t="s" s="11">
         <v>17</v>
-      </c>
-      <c r="J2" t="s" s="11">
-        <v>18</v>
       </c>
     </row>
     <row r="3">
       <c r="B3" t="s" s="12">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s" s="13">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="D3" t="s" s="14">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="E3" t="s" s="15">
         <v>13</v>
@@ -18476,21 +18627,21 @@
         <v>14</v>
       </c>
       <c r="I3" t="s" s="19">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J3" t="s" s="20">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4">
       <c r="B4" t="s" s="21">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s" s="22">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="D4" t="s" s="23">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="E4" t="s" s="24">
         <v>13</v>
@@ -18505,21 +18656,21 @@
         <v>14</v>
       </c>
       <c r="I4" t="s" s="28">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J4" t="s" s="29">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="s" s="30">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C5" t="s" s="31">
         <v>11</v>
       </c>
       <c r="D5" t="s" s="32">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E5" t="s" s="33">
         <v>13</v>
@@ -18534,21 +18685,21 @@
         <v>14</v>
       </c>
       <c r="I5" t="s" s="37">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J5" t="s" s="38">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="s" s="39">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s" s="40">
         <v>11</v>
       </c>
       <c r="D6" t="s" s="41">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E6" t="s" s="42">
         <v>13</v>
@@ -18563,21 +18714,21 @@
         <v>14</v>
       </c>
       <c r="I6" t="s" s="46">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J6" t="s" s="47">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="s" s="48">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C7" t="s" s="49">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="D7" t="s" s="50">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E7" t="s" s="51">
         <v>13</v>
@@ -18592,10 +18743,300 @@
         <v>14</v>
       </c>
       <c r="I7" t="s" s="55">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J7" t="s" s="56">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="s" s="57">
+        <v>23</v>
+      </c>
+      <c r="C8" t="s" s="58">
+        <v>11</v>
+      </c>
+      <c r="D8" t="s" s="59">
+        <v>28</v>
+      </c>
+      <c r="E8" t="s" s="60">
+        <v>13</v>
+      </c>
+      <c r="F8" t="s" s="61">
         <v>14</v>
+      </c>
+      <c r="G8" t="s" s="62">
+        <v>15</v>
+      </c>
+      <c r="H8" t="s" s="63">
+        <v>14</v>
+      </c>
+      <c r="I8" t="s" s="64">
+        <v>16</v>
+      </c>
+      <c r="J8" t="s" s="65">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="s" s="66">
+        <v>30</v>
+      </c>
+      <c r="C9" t="s" s="67">
+        <v>11</v>
+      </c>
+      <c r="D9" t="s" s="68">
+        <v>31</v>
+      </c>
+      <c r="E9" t="s" s="69">
+        <v>13</v>
+      </c>
+      <c r="F9" t="s" s="70">
+        <v>14</v>
+      </c>
+      <c r="G9" t="s" s="71">
+        <v>15</v>
+      </c>
+      <c r="H9" t="s" s="72">
+        <v>14</v>
+      </c>
+      <c r="I9" t="s" s="73">
+        <v>16</v>
+      </c>
+      <c r="J9" t="s" s="74">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="s" s="75">
+        <v>33</v>
+      </c>
+      <c r="C10" t="s" s="76">
+        <v>11</v>
+      </c>
+      <c r="D10" t="s" s="77">
+        <v>34</v>
+      </c>
+      <c r="E10" t="s" s="78">
+        <v>13</v>
+      </c>
+      <c r="F10" t="s" s="79">
+        <v>14</v>
+      </c>
+      <c r="G10" t="s" s="80">
+        <v>15</v>
+      </c>
+      <c r="H10" t="s" s="81">
+        <v>14</v>
+      </c>
+      <c r="I10" t="s" s="82">
+        <v>16</v>
+      </c>
+      <c r="J10" t="s" s="83">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="s" s="84">
+        <v>33</v>
+      </c>
+      <c r="C11" t="s" s="85">
+        <v>11</v>
+      </c>
+      <c r="D11" t="s" s="86">
+        <v>36</v>
+      </c>
+      <c r="E11" t="s" s="87">
+        <v>13</v>
+      </c>
+      <c r="F11" t="s" s="88">
+        <v>14</v>
+      </c>
+      <c r="G11" t="s" s="89">
+        <v>15</v>
+      </c>
+      <c r="H11" t="s" s="90">
+        <v>14</v>
+      </c>
+      <c r="I11" t="s" s="91">
+        <v>16</v>
+      </c>
+      <c r="J11" t="s" s="92">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="s" s="93">
+        <v>33</v>
+      </c>
+      <c r="C12" t="s" s="94">
+        <v>11</v>
+      </c>
+      <c r="D12" t="s" s="95">
+        <v>38</v>
+      </c>
+      <c r="E12" t="s" s="96">
+        <v>13</v>
+      </c>
+      <c r="F12" t="s" s="97">
+        <v>14</v>
+      </c>
+      <c r="G12" t="s" s="98">
+        <v>15</v>
+      </c>
+      <c r="H12" t="s" s="99">
+        <v>14</v>
+      </c>
+      <c r="I12" t="s" s="100">
+        <v>16</v>
+      </c>
+      <c r="J12" t="s" s="101">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="s" s="102">
+        <v>40</v>
+      </c>
+      <c r="C13" t="s" s="103">
+        <v>11</v>
+      </c>
+      <c r="D13" t="s" s="104">
+        <v>41</v>
+      </c>
+      <c r="E13" t="s" s="105">
+        <v>13</v>
+      </c>
+      <c r="F13" t="s" s="106">
+        <v>14</v>
+      </c>
+      <c r="G13" t="s" s="107">
+        <v>15</v>
+      </c>
+      <c r="H13" t="s" s="108">
+        <v>14</v>
+      </c>
+      <c r="I13" t="s" s="109">
+        <v>16</v>
+      </c>
+      <c r="J13" t="s" s="110">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="s" s="111">
+        <v>33</v>
+      </c>
+      <c r="C14" t="s" s="112">
+        <v>11</v>
+      </c>
+      <c r="D14" t="s" s="113">
+        <v>43</v>
+      </c>
+      <c r="E14" t="s" s="114">
+        <v>13</v>
+      </c>
+      <c r="F14" t="s" s="115">
+        <v>14</v>
+      </c>
+      <c r="G14" t="s" s="116">
+        <v>15</v>
+      </c>
+      <c r="H14" t="s" s="117">
+        <v>14</v>
+      </c>
+      <c r="I14" t="s" s="118">
+        <v>16</v>
+      </c>
+      <c r="J14" t="s" s="119">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="s" s="120">
+        <v>33</v>
+      </c>
+      <c r="C15" t="s" s="121">
+        <v>11</v>
+      </c>
+      <c r="D15" t="s" s="122">
+        <v>45</v>
+      </c>
+      <c r="E15" t="s" s="123">
+        <v>13</v>
+      </c>
+      <c r="F15" t="s" s="124">
+        <v>14</v>
+      </c>
+      <c r="G15" t="s" s="125">
+        <v>15</v>
+      </c>
+      <c r="H15" t="s" s="126">
+        <v>14</v>
+      </c>
+      <c r="I15" t="s" s="127">
+        <v>16</v>
+      </c>
+      <c r="J15" t="s" s="128">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="s" s="129">
+        <v>33</v>
+      </c>
+      <c r="C16" t="s" s="130">
+        <v>11</v>
+      </c>
+      <c r="D16" t="s" s="131">
+        <v>47</v>
+      </c>
+      <c r="E16" t="s" s="132">
+        <v>13</v>
+      </c>
+      <c r="F16" t="s" s="133">
+        <v>14</v>
+      </c>
+      <c r="G16" t="s" s="134">
+        <v>15</v>
+      </c>
+      <c r="H16" t="s" s="135">
+        <v>14</v>
+      </c>
+      <c r="I16" t="s" s="136">
+        <v>16</v>
+      </c>
+      <c r="J16" t="s" s="137">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="s" s="138">
+        <v>33</v>
+      </c>
+      <c r="C17" t="s" s="139">
+        <v>11</v>
+      </c>
+      <c r="D17" t="s" s="140">
+        <v>49</v>
+      </c>
+      <c r="E17" t="s" s="141">
+        <v>13</v>
+      </c>
+      <c r="F17" t="s" s="142">
+        <v>14</v>
+      </c>
+      <c r="G17" t="s" s="143">
+        <v>15</v>
+      </c>
+      <c r="H17" t="s" s="144">
+        <v>14</v>
+      </c>
+      <c r="I17" t="s" s="145">
+        <v>16</v>
+      </c>
+      <c r="J17" t="s" s="146">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>